<commit_message>
Aggiornato dizionario e attivazione tempo iniziale di avvio programmabile
</commit_message>
<xml_diff>
--- a/Resources/Dizionari STEM.xlsx
+++ b/Resources/Dizionari STEM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michele\Nextcloud\PROTOCOLLO STEM\Protocollo di comunicazione STEM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michele\OneDrive\Dati\Lavoro\VSProjects\StemProtocolCompanion\bin\publish\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675AAF32-33AE-4229-8299-5498AF11CBE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E05573-7C8A-48DD-BE5D-B0042C1FA5B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="500" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COMANDI" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2938" uniqueCount="925">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2951" uniqueCount="931">
   <si>
     <t>NOME COMANDO</t>
   </si>
@@ -3593,6 +3593,24 @@
   </si>
   <si>
     <t>temperatura interna al micro in gradi</t>
+  </si>
+  <si>
+    <t>Gateway loading file</t>
+  </si>
+  <si>
+    <t>Gateway loading file size</t>
+  </si>
+  <si>
+    <t>Gateway loading file transfered</t>
+  </si>
+  <si>
+    <t>Gateway firmware version</t>
+  </si>
+  <si>
+    <t>Tempo di ritardo all'accensione</t>
+  </si>
+  <si>
+    <t>Tempo in ms di ritardo all'accensione</t>
   </si>
 </sst>
 </file>
@@ -12361,9 +12379,9 @@
   <dimension ref="A1:AMM125"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35" style="3" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -15295,8 +15313,8 @@
       <c r="T47" s="3"/>
     </row>
     <row r="48" spans="1:1027" x14ac:dyDescent="0.25">
-      <c r="A48" s="85" t="s">
-        <v>786</v>
+      <c r="A48" s="41" t="s">
+        <v>929</v>
       </c>
       <c r="B48" s="3">
         <v>80</v>
@@ -15305,15 +15323,24 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D48" s="3"/>
+      <c r="D48" s="3" t="s">
+        <v>241</v>
+      </c>
       <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
+      <c r="F48" s="3">
+        <v>0</v>
+      </c>
+      <c r="G48" s="3">
+        <v>65535</v>
+      </c>
       <c r="H48" s="3"/>
       <c r="I48" s="3" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="J48" s="3"/>
+      <c r="K48" s="3" t="s">
+        <v>930</v>
+      </c>
       <c r="L48" s="3"/>
       <c r="M48" s="3"/>
       <c r="N48" s="3"/>
@@ -40907,7 +40934,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2D0C0CD-5519-46B2-A9F3-B4381168B0E7}">
-  <dimension ref="A1:W67"/>
+  <dimension ref="A1:W71"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.7109375" style="3" customWidth="1"/>
@@ -42873,6 +42900,65 @@
       </c>
       <c r="D67" s="3" t="s">
         <v>141</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="41" t="s">
+        <v>925</v>
+      </c>
+      <c r="B68" s="3">
+        <v>80</v>
+      </c>
+      <c r="C68" s="3">
+        <v>19</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="41" t="s">
+        <v>926</v>
+      </c>
+      <c r="B69" s="3">
+        <v>80</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="41" t="s">
+        <v>927</v>
+      </c>
+      <c r="B70" s="3">
+        <v>80</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="41" t="s">
+        <v>928</v>
+      </c>
+      <c r="B71" s="3">
+        <v>80</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="E71" s="95">
+        <v>255255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Attivazione di tutti i parametri. Necessita di firmware versione 1.21
</commit_message>
<xml_diff>
--- a/Resources/Dizionari STEM.xlsx
+++ b/Resources/Dizionari STEM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michele\OneDrive\Dati\Lavoro\VSProjects\StemProtocolCompanion\bin\publish\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michele\Nextcloud\PROTOCOLLO STEM\Protocollo di comunicazione STEM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E05573-7C8A-48DD-BE5D-B0042C1FA5B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22853CDB-3FDB-4F88-8281-F00F00C34A99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="500" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-2340" yWindow="-16320" windowWidth="29040" windowHeight="15840" tabRatio="500" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COMANDI" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2951" uniqueCount="931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2968" uniqueCount="937">
   <si>
     <t>NOME COMANDO</t>
   </si>
@@ -3611,6 +3611,25 @@
   </si>
   <si>
     <t>Tempo in ms di ritardo all'accensione</t>
+  </si>
+  <si>
+    <t>Posizione tastiera</t>
+  </si>
+  <si>
+    <t>0 = destra (default)
+1 =  sinistra</t>
+  </si>
+  <si>
+    <t>Altezza di carico</t>
+  </si>
+  <si>
+    <t>Altezza 1 da chiuso</t>
+  </si>
+  <si>
+    <t>Altezza 2 da chiuso</t>
+  </si>
+  <si>
+    <t>Altezza 3 da chiuso</t>
   </si>
 </sst>
 </file>
@@ -16122,8 +16141,8 @@
       <c r="T72" s="3"/>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A73" s="46" t="s">
-        <v>347</v>
+      <c r="A73" s="41" t="s">
+        <v>933</v>
       </c>
       <c r="B73" s="3">
         <v>80</v>
@@ -16132,12 +16151,22 @@
         <f t="shared" si="0"/>
         <v>2B</v>
       </c>
-      <c r="D73" s="3"/>
+      <c r="D73" s="3" t="s">
+        <v>241</v>
+      </c>
       <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="3"/>
-      <c r="H73" s="3"/>
-      <c r="I73" s="3"/>
+      <c r="F73" s="3">
+        <v>0</v>
+      </c>
+      <c r="G73" s="3">
+        <v>65535</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="I73" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="J73" s="3"/>
       <c r="L73" s="3"/>
       <c r="M73" s="3"/>
@@ -16150,8 +16179,8 @@
       <c r="T73" s="3"/>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A74" s="46" t="s">
-        <v>347</v>
+      <c r="A74" s="41" t="s">
+        <v>934</v>
       </c>
       <c r="B74" s="3">
         <v>80</v>
@@ -16160,12 +16189,22 @@
         <f t="shared" si="0"/>
         <v>2C</v>
       </c>
-      <c r="D74" s="3"/>
+      <c r="D74" s="3" t="s">
+        <v>241</v>
+      </c>
       <c r="E74" s="3"/>
-      <c r="F74" s="3"/>
-      <c r="G74" s="3"/>
-      <c r="H74" s="3"/>
-      <c r="I74" s="3"/>
+      <c r="F74" s="3">
+        <v>0</v>
+      </c>
+      <c r="G74" s="3">
+        <v>65535</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="J74" s="3"/>
       <c r="L74" s="3"/>
       <c r="M74" s="3"/>
@@ -16178,8 +16217,8 @@
       <c r="T74" s="3"/>
     </row>
     <row r="75" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A75" s="46" t="s">
-        <v>347</v>
+      <c r="A75" s="41" t="s">
+        <v>935</v>
       </c>
       <c r="B75" s="3">
         <v>80</v>
@@ -16188,12 +16227,22 @@
         <f t="shared" si="0"/>
         <v>2D</v>
       </c>
-      <c r="D75" s="3"/>
+      <c r="D75" s="3" t="s">
+        <v>241</v>
+      </c>
       <c r="E75" s="3"/>
-      <c r="F75" s="3"/>
-      <c r="G75" s="3"/>
-      <c r="H75" s="3"/>
-      <c r="I75" s="3"/>
+      <c r="F75" s="3">
+        <v>0</v>
+      </c>
+      <c r="G75" s="3">
+        <v>65535</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="J75" s="3"/>
       <c r="L75" s="3"/>
       <c r="M75" s="3"/>
@@ -16206,8 +16255,8 @@
       <c r="T75" s="3"/>
     </row>
     <row r="76" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A76" s="46" t="s">
-        <v>347</v>
+      <c r="A76" s="41" t="s">
+        <v>936</v>
       </c>
       <c r="B76" s="3">
         <v>80</v>
@@ -16216,12 +16265,22 @@
         <f t="shared" si="0"/>
         <v>2E</v>
       </c>
-      <c r="D76" s="3"/>
+      <c r="D76" s="3" t="s">
+        <v>241</v>
+      </c>
       <c r="E76" s="3"/>
-      <c r="F76" s="3"/>
-      <c r="G76" s="3"/>
-      <c r="H76" s="3"/>
-      <c r="I76" s="3"/>
+      <c r="F76" s="3">
+        <v>0</v>
+      </c>
+      <c r="G76" s="3">
+        <v>65535</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>643</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="J76" s="3"/>
       <c r="L76" s="3"/>
       <c r="M76" s="3"/>
@@ -25368,15 +25427,44 @@
       <c r="T27" s="3"/>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
+      <c r="A28" s="41" t="str">
+        <f>IF('DATI LOGICI'!A26&lt;&gt;"",'DATI LOGICI'!A26,"")</f>
+        <v>Firmware Bootloader</v>
+      </c>
+      <c r="B28" s="3">
+        <f>IF('DATI LOGICI'!B26&lt;&gt;"",'DATI LOGICI'!B26,"")</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="3">
+        <f>IF('DATI LOGICI'!C26&lt;&gt;"",'DATI LOGICI'!C26,"")</f>
+        <v>17</v>
+      </c>
+      <c r="D28" s="3" t="str">
+        <f>IF('DATI LOGICI'!D26&lt;&gt;"",'DATI LOGICI'!D26,"")</f>
+        <v xml:space="preserve">uint16_t </v>
+      </c>
+      <c r="E28" s="3" t="str">
+        <f>IF('DATI LOGICI'!E26&lt;&gt;"",'DATI LOGICI'!E26,"")</f>
+        <v>255.255</v>
+      </c>
+      <c r="F28" s="3">
+        <f>IF('DATI LOGICI'!F26&lt;&gt;"",'DATI LOGICI'!F26,"")</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="3" t="str">
+        <f>IF('DATI LOGICI'!G26&lt;&gt;"",'DATI LOGICI'!G26,"")</f>
+        <v>255.255</v>
+      </c>
+      <c r="H28" s="3" t="str">
+        <f>IF('DATI LOGICI'!H26&lt;&gt;"",'DATI LOGICI'!H26,"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="3" t="str">
+        <f>IF('DATI LOGICI'!I26&lt;&gt;"",'DATI LOGICI'!I26,"")</f>
+        <v>R</v>
+      </c>
       <c r="J28" s="3"/>
+      <c r="K28" s="10"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
       <c r="N28" s="3"/>
@@ -31730,7 +31818,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AMM53"/>
+  <dimension ref="A1:AMM54"/>
   <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="60.7109375" style="1" customWidth="1"/>
@@ -33176,6 +33264,32 @@
       <c r="L53" s="21"/>
       <c r="M53" s="21"/>
       <c r="N53" s="21"/>
+    </row>
+    <row r="54" spans="1:14 1027:1027" ht="30" x14ac:dyDescent="0.25">
+      <c r="A54" s="19" t="s">
+        <v>931</v>
+      </c>
+      <c r="B54" s="3">
+        <v>80</v>
+      </c>
+      <c r="C54" s="3">
+        <v>45</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="J54" s="10" t="s">
+        <v>932</v>
+      </c>
+      <c r="K54" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="L54" s="21"/>
+      <c r="M54" s="21"/>
+      <c r="N54" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>